<commit_message>
Collapse the advanced columns of a form workbook's Fields sheet
The template builder grouped the advanced columns with Group(true), which marks the group
collapsed but leaves its columns visible, so Excel and LibreOffice opened the workbook with
every advanced column expanded. Hide the grouped columns as well and regenerate both templates.
</commit_message>
<xml_diff>
--- a/tools/Polhem.Definition.Spreadsheet/Templates/FormSchema.en.xlsx
+++ b/tools/Polhem.Definition.Spreadsheet/Templates/FormSchema.en.xlsx
@@ -2359,11 +2359,11 @@
     <x:col min="14" max="15" width="28.710625" style="0" customWidth="1"/>
     <x:col min="16" max="17" width="14.710625" style="0" customWidth="1"/>
     <x:col min="18" max="18" width="10.710625" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="14.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="20" max="20" width="24.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="21" max="24" width="14.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="25" max="25" width="28.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="26" max="29" width="14.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="19" max="19" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="20" max="20" width="24.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="21" max="24" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="25" max="25" width="28.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="26" max="29" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:29">

</xml_diff>

<commit_message>
Collapse the advanced columns of a form workbook's Fields sheet (#131)
The template builder grouped the advanced columns with Group(true), which marks the group
collapsed but leaves its columns visible, so Excel and LibreOffice opened the workbook with
every advanced column expanded. Hide the grouped columns as well and regenerate both templates.
</commit_message>
<xml_diff>
--- a/tools/Polhem.Definition.Spreadsheet/Templates/FormSchema.en.xlsx
+++ b/tools/Polhem.Definition.Spreadsheet/Templates/FormSchema.en.xlsx
@@ -2359,11 +2359,11 @@
     <x:col min="14" max="15" width="28.710625" style="0" customWidth="1"/>
     <x:col min="16" max="17" width="14.710625" style="0" customWidth="1"/>
     <x:col min="18" max="18" width="10.710625" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="14.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="20" max="20" width="24.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="21" max="24" width="14.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="25" max="25" width="28.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="26" max="29" width="14.710625" style="0" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="19" max="19" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="20" max="20" width="24.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="21" max="24" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="25" max="25" width="28.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="26" max="29" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:29">

</xml_diff>

<commit_message>
Pin FieldValueChange's access control and give it a workbook column
CI found two gates the new member has to pass:

- ApiAccessControlPinTests pins every action's declaration; it now lists
  FormBusinessObject.FieldValueChange as Public / Authenticated, the same
  declaration the BO surface baseline already records.
- FormWorkbookCoverageTests requires a workbook column for every serialized
  FormField property, so ValueChangeCallback gets an advanced Y/N column
  ("Server callback on change" / 異動時回呼後端) and the English and zh-TW
  form templates are regenerated.
</commit_message>
<xml_diff>
--- a/tools/Polhem.Definition.Spreadsheet/Templates/FormSchema.en.xlsx
+++ b/tools/Polhem.Definition.Spreadsheet/Templates/FormSchema.en.xlsx
@@ -531,6 +531,15 @@
     <x:t>DisplayFields</x:t>
   </x:si>
   <x:si>
+    <x:t>Server callback on change</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ValueChangeCallback</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Y asks the server for related values or validation when the value changes.</x:t>
+  </x:si>
+  <x:si>
     <x:t>Language enum</x:t>
   </x:si>
   <x:si>
@@ -733,6 +742,9 @@
   </x:si>
   <x:si>
     <x:t>{{Fields.DisplayFields}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{Fields.ValueChangeCallback}}</x:t>
   </x:si>
   <x:si>
     <x:t>{{Fields.LangEnumName}}</x:t>
@@ -1173,7 +1185,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D65"/>
+  <x:dimension ref="A1:D66"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="12.710625" style="0" customWidth="1"/>
@@ -1831,7 +1843,7 @@
         <x:v>171</x:v>
       </x:c>
       <x:c r="D54" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:4">
@@ -1839,10 +1851,10 @@
         <x:v>115</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C55" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="D55" s="0" t="s">
         <x:v>57</x:v>
@@ -1853,10 +1865,10 @@
         <x:v>115</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C56" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D56" s="0" t="s">
         <x:v>57</x:v>
@@ -1864,13 +1876,13 @@
     </x:row>
     <x:row r="57" spans="1:4">
       <x:c r="A57" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="C57" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D57" s="0" t="s">
         <x:v>57</x:v>
@@ -1878,38 +1890,38 @@
     </x:row>
     <x:row r="58" spans="1:4">
       <x:c r="A58" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C58" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="D58" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:4">
       <x:c r="A59" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>180</x:v>
       </x:c>
       <x:c r="C59" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D59" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:4">
       <x:c r="A60" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="C60" s="0" t="s">
         <x:v>183</x:v>
@@ -1920,7 +1932,7 @@
     </x:row>
     <x:row r="61" spans="1:4">
       <x:c r="A61" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
         <x:v>185</x:v>
@@ -1934,7 +1946,7 @@
     </x:row>
     <x:row r="62" spans="1:4">
       <x:c r="A62" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B62" s="0" t="s">
         <x:v>188</x:v>
@@ -1943,18 +1955,18 @@
         <x:v>189</x:v>
       </x:c>
       <x:c r="D62" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:4">
       <x:c r="A63" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B63" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="C63" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D63" s="0" t="s">
         <x:v>57</x:v>
@@ -1962,29 +1974,43 @@
     </x:row>
     <x:row r="64" spans="1:4">
       <x:c r="A64" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="C64" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="D64" s="0" t="s">
-        <x:v>193</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:4">
       <x:c r="A65" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B65" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="C65" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D65" s="0" t="s">
+        <x:v>196</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" spans="1:4">
+      <x:c r="A66" s="0" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B66" s="0" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="C66" s="0" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="D66" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
     </x:row>
@@ -2013,11 +2039,11 @@
   <x:sheetData>
     <x:row r="1" spans="1:4">
       <x:c r="A1" s="2" t="s">
-        <x:v>195</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2" t="s">
-        <x:v>196</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
         <x:v>68</x:v>
@@ -2031,7 +2057,7 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>72</x:v>
@@ -2045,7 +2071,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
         <x:v>75</x:v>
@@ -2059,7 +2085,7 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>199</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
         <x:v>78</x:v>
@@ -2073,7 +2099,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>200</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
         <x:v>80</x:v>
@@ -2087,7 +2113,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
         <x:v>83</x:v>
@@ -2101,7 +2127,7 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
         <x:v>86</x:v>
@@ -2115,7 +2141,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>203</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
         <x:v>89</x:v>
@@ -2129,7 +2155,7 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
         <x:v>92</x:v>
@@ -2143,7 +2169,7 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
         <x:v>95</x:v>
@@ -2157,7 +2183,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>206</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
         <x:v>98</x:v>
@@ -2171,7 +2197,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>207</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
         <x:v>101</x:v>
@@ -2185,7 +2211,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>208</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
         <x:v>104</x:v>
@@ -2199,7 +2225,7 @@
         <x:v>106</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>209</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
         <x:v>107</x:v>
@@ -2268,16 +2294,16 @@
     </x:row>
     <x:row r="3" spans="1:4">
       <x:c r="A3" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>212</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>213</x:v>
+        <x:v>216</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2294,7 +2320,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:AA3"/>
+  <x:dimension ref="A1:AB3"/>
   <x:sheetFormatPr defaultRowHeight="15" outlineLevelCol="1"/>
   <x:cols>
     <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
@@ -2312,10 +2338,12 @@
     <x:col min="18" max="18" width="10.710625" style="0" customWidth="1"/>
     <x:col min="19" max="19" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
     <x:col min="20" max="20" width="24.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <x:col min="21" max="27" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="21" max="24" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="25" max="25" width="8.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <x:col min="26" max="28" width="14.710625" style="0" hidden="1" customWidth="1" outlineLevel="1" collapsed="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:27">
+    <x:row r="1" spans="1:28">
       <x:c r="A1" s="2" t="s">
         <x:v>116</x:v>
       </x:c>
@@ -2392,13 +2420,16 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="Z1" s="4" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="AA1" s="4" t="s">
-        <x:v>173</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:27" hidden="1">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="AB1" s="4" t="s">
+        <x:v>176</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:28" hidden="1">
       <x:c r="A2" s="0" t="s">
         <x:v>110</x:v>
       </x:c>
@@ -2475,93 +2506,99 @@
         <x:v>171</x:v>
       </x:c>
       <x:c r="Z2" s="0" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="AA2" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="AA2" s="0" t="s">
+      <x:c r="AB2" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:27">
+    <x:row r="3" spans="1:28">
       <x:c r="A3" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>216</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>217</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>218</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>219</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>220</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>221</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>222</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="J3" s="0" t="s">
-        <x:v>223</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="K3" s="0" t="s">
-        <x:v>224</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="L3" s="0" t="s">
-        <x:v>225</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
-        <x:v>226</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="N3" s="0" t="s">
-        <x:v>227</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="O3" s="0" t="s">
-        <x:v>228</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="P3" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="Q3" s="0" t="s">
-        <x:v>230</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="R3" s="0" t="s">
-        <x:v>231</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="S3" s="0" t="s">
-        <x:v>232</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="T3" s="0" t="s">
-        <x:v>233</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="U3" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="V3" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="W3" s="0" t="s">
-        <x:v>236</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="X3" s="0" t="s">
-        <x:v>237</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="Y3" s="0" t="s">
-        <x:v>238</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="Z3" s="0" t="s">
-        <x:v>239</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="AA3" s="0" t="s">
-        <x:v>240</x:v>
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="AB3" s="0" t="s">
+        <x:v>244</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2583,7 +2620,7 @@
           <x14:formula1>
             <xm:f>Lists!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G3:I1000</xm:sqref>
+          <xm:sqref>G3:I1000 Y3:Y1000</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
           <x14:formula1>
@@ -2607,13 +2644,13 @@
           <x14:formula1>
             <xm:f>Lists!$G$2:$G$4</xm:f>
           </x14:formula1>
-          <xm:sqref>Z3:Z1000</xm:sqref>
+          <xm:sqref>AA3:AA1000</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
           <x14:formula1>
             <xm:f>Lists!$H$2:$H$5</xm:f>
           </x14:formula1>
-          <xm:sqref>AA3:AA1000</xm:sqref>
+          <xm:sqref>AB3:AB1000</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </x:ext>
@@ -2641,89 +2678,89 @@
   <x:sheetData>
     <x:row r="1" spans="1:9">
       <x:c r="A1" s="2" t="s">
-        <x:v>175</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B1" s="2" t="s">
-        <x:v>177</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C1" s="2" t="s">
-        <x:v>180</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D1" s="2" t="s">
-        <x:v>182</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E1" s="2" t="s">
-        <x:v>185</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="F1" s="2" t="s">
-        <x:v>188</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="G1" s="2" t="s">
-        <x:v>190</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="H1" s="2" t="s">
-        <x:v>192</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="I1" s="2" t="s">
-        <x:v>194</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:9" hidden="1">
       <x:c r="A2" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>186</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>189</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
       <x:c r="A3" s="0" t="s">
-        <x:v>241</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>242</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>243</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>244</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>245</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>248</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>249</x:v>
+        <x:v>253</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>